<commit_message>
Data associated with this study.
</commit_message>
<xml_diff>
--- a/HAB_MCC_DOC_Dates_Data/Kisumu Bay Data.xlsx
+++ b/HAB_MCC_DOC_Dates_Data/Kisumu Bay Data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okomojacob/Documents/📚Research &amp; Academia/Final Publication 2025/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okomojacob/Documents/📚Research &amp; Academia/Final Publication 2025/FinalYearProject/HAB_MCC_DOC_Dates_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{099F4A52-B481-D74D-8F62-7F72E2E5C2BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D102F31-C2A3-B24B-B589-37352AFAB624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28800" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{C80561F6-58AE-47CB-82DA-A3E0AB24ED8B}"/>
   </bookViews>
@@ -257,7 +257,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -304,7 +304,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -316,10 +316,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -816,19 +813,19 @@
       <c r="H5" s="3">
         <v>39.96</v>
       </c>
-      <c r="I5" s="21" t="s">
+      <c r="I5" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J5" s="21">
+      <c r="J5" s="15">
         <v>26.3</v>
       </c>
-      <c r="K5" s="21">
+      <c r="K5" s="15">
         <v>25.3</v>
       </c>
-      <c r="L5" s="21">
+      <c r="L5" s="15">
         <v>18</v>
       </c>
-      <c r="M5" s="21">
+      <c r="M5" s="15">
         <v>4.3</v>
       </c>
     </row>
@@ -1432,19 +1429,19 @@
       <c r="H23" s="14">
         <v>9.92</v>
       </c>
-      <c r="I23" s="21" t="s">
+      <c r="I23" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J23" s="21">
+      <c r="J23" s="15">
         <v>2.87</v>
       </c>
       <c r="K23" s="20">
         <v>19.38</v>
       </c>
-      <c r="L23" s="21">
+      <c r="L23" s="15">
         <v>2.7</v>
       </c>
-      <c r="M23" s="21">
+      <c r="M23" s="15">
         <v>16.600000000000001</v>
       </c>
     </row>
@@ -1471,13 +1468,13 @@
       <c r="H24" s="14">
         <v>13.4</v>
       </c>
-      <c r="I24" s="21"/>
-      <c r="J24" s="21"/>
-      <c r="K24" s="21"/>
-      <c r="L24" s="21">
+      <c r="I24" s="15"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="15"/>
+      <c r="L24" s="15">
         <v>4</v>
       </c>
-      <c r="M24" s="21">
+      <c r="M24" s="15">
         <v>0.09</v>
       </c>
     </row>
@@ -1504,19 +1501,19 @@
       <c r="H25" s="14">
         <v>10.210000000000001</v>
       </c>
-      <c r="I25" s="21" t="s">
+      <c r="I25" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J25" s="21">
+      <c r="J25" s="15">
         <v>21.2</v>
       </c>
-      <c r="K25" s="21">
+      <c r="K25" s="15">
         <v>30.6</v>
       </c>
-      <c r="L25" s="21">
+      <c r="L25" s="15">
         <v>23</v>
       </c>
-      <c r="M25" s="21">
+      <c r="M25" s="15">
         <v>7.7</v>
       </c>
     </row>
@@ -1543,19 +1540,19 @@
       <c r="H26" s="14">
         <v>12.96</v>
       </c>
-      <c r="I26" s="21" t="s">
+      <c r="I26" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J26" s="21">
+      <c r="J26" s="15">
         <v>22.8</v>
       </c>
-      <c r="K26" s="21">
+      <c r="K26" s="15">
         <v>23.8888</v>
       </c>
-      <c r="L26" s="21">
+      <c r="L26" s="15">
         <v>7</v>
       </c>
-      <c r="M26" s="21">
+      <c r="M26" s="15">
         <v>1.1000000000000001</v>
       </c>
     </row>
@@ -1582,17 +1579,17 @@
       <c r="H27" s="14">
         <v>751.95</v>
       </c>
-      <c r="I27" s="21"/>
-      <c r="J27" s="21">
+      <c r="I27" s="15"/>
+      <c r="J27" s="15">
         <v>12.9</v>
       </c>
-      <c r="K27" s="21">
+      <c r="K27" s="15">
         <v>17.600000000000001</v>
       </c>
-      <c r="L27" s="21">
+      <c r="L27" s="15">
         <v>6.5</v>
       </c>
-      <c r="M27" s="21">
+      <c r="M27" s="15">
         <v>0.7</v>
       </c>
     </row>
@@ -1619,17 +1616,17 @@
       <c r="H28" s="14">
         <v>23.58</v>
       </c>
-      <c r="I28" s="21" t="s">
+      <c r="I28" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J28" s="21">
+      <c r="J28" s="15">
         <v>23.2</v>
       </c>
-      <c r="K28" s="21"/>
-      <c r="L28" s="21">
+      <c r="K28" s="15"/>
+      <c r="L28" s="15">
         <v>8.1999999999999993</v>
       </c>
-      <c r="M28" s="21">
+      <c r="M28" s="15">
         <v>0.4</v>
       </c>
     </row>
@@ -1656,19 +1653,19 @@
       <c r="H29" s="14">
         <v>11.52</v>
       </c>
-      <c r="I29" s="21" t="s">
+      <c r="I29" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J29" s="21">
+      <c r="J29" s="15">
         <v>24.2</v>
       </c>
-      <c r="K29" s="21">
+      <c r="K29" s="15">
         <v>19.2</v>
       </c>
-      <c r="L29" s="21">
+      <c r="L29" s="15">
         <v>16.73</v>
       </c>
-      <c r="M29" s="21">
+      <c r="M29" s="15">
         <v>5.3</v>
       </c>
     </row>
@@ -1697,19 +1694,19 @@
       <c r="H30" s="14">
         <v>53.42</v>
       </c>
-      <c r="I30" s="21" t="s">
+      <c r="I30" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J30" s="21">
+      <c r="J30" s="15">
         <v>23.7</v>
       </c>
-      <c r="K30" s="21">
+      <c r="K30" s="15">
         <v>25.6</v>
       </c>
-      <c r="L30" s="21">
+      <c r="L30" s="15">
         <v>17.7</v>
       </c>
-      <c r="M30" s="21">
+      <c r="M30" s="15">
         <v>4.3</v>
       </c>
     </row>
@@ -1738,19 +1735,19 @@
       <c r="H31" s="14">
         <v>38.729999999999997</v>
       </c>
-      <c r="I31" s="21" t="s">
+      <c r="I31" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J31" s="21">
+      <c r="J31" s="15">
         <v>9.8000000000000007</v>
       </c>
-      <c r="K31" s="21">
+      <c r="K31" s="15">
         <v>11.8</v>
       </c>
-      <c r="L31" s="21">
+      <c r="L31" s="15">
         <v>6.9</v>
       </c>
-      <c r="M31" s="21">
+      <c r="M31" s="15">
         <v>2.2999999999999998</v>
       </c>
     </row>
@@ -1779,17 +1776,17 @@
       <c r="H32" s="14">
         <v>24.36</v>
       </c>
-      <c r="I32" s="21" t="s">
+      <c r="I32" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J32" s="21"/>
-      <c r="K32" s="21">
+      <c r="J32" s="15"/>
+      <c r="K32" s="15">
         <v>10.3</v>
       </c>
-      <c r="L32" s="21">
+      <c r="L32" s="15">
         <v>11.4</v>
       </c>
-      <c r="M32" s="21">
+      <c r="M32" s="15">
         <v>0.9</v>
       </c>
     </row>
@@ -1818,19 +1815,19 @@
       <c r="H33" s="14">
         <v>33.049999999999997</v>
       </c>
-      <c r="I33" s="21" t="s">
+      <c r="I33" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J33" s="21">
+      <c r="J33" s="15">
         <v>18.600000000000001</v>
       </c>
-      <c r="K33" s="21">
+      <c r="K33" s="15">
         <v>18.1111</v>
       </c>
-      <c r="L33" s="21">
+      <c r="L33" s="15">
         <v>19.3</v>
       </c>
-      <c r="M33" s="21"/>
+      <c r="M33" s="15"/>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="1"/>
@@ -1841,11 +1838,11 @@
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
-      <c r="I34" s="21"/>
-      <c r="J34" s="21"/>
-      <c r="K34" s="21"/>
-      <c r="L34" s="21"/>
-      <c r="M34" s="21"/>
+      <c r="I34" s="15"/>
+      <c r="J34" s="15"/>
+      <c r="K34" s="15"/>
+      <c r="L34" s="15"/>
+      <c r="M34" s="15"/>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
@@ -1868,19 +1865,19 @@
       <c r="H35" s="3">
         <v>254.32</v>
       </c>
-      <c r="I35" s="21" t="s">
+      <c r="I35" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J35" s="21">
+      <c r="J35" s="15">
         <v>26.3</v>
       </c>
-      <c r="K35" s="21">
+      <c r="K35" s="15">
         <v>21</v>
       </c>
-      <c r="L35" s="21">
+      <c r="L35" s="15">
         <v>12.7</v>
       </c>
-      <c r="M35" s="21">
+      <c r="M35" s="15">
         <v>6.4</v>
       </c>
     </row>
@@ -1907,15 +1904,15 @@
       <c r="H36" s="3">
         <v>8.41</v>
       </c>
-      <c r="I36" s="21"/>
-      <c r="J36" s="21">
+      <c r="I36" s="15"/>
+      <c r="J36" s="15">
         <v>19.3</v>
       </c>
-      <c r="K36" s="21">
+      <c r="K36" s="15">
         <v>26.4</v>
       </c>
-      <c r="L36" s="21"/>
-      <c r="M36" s="21">
+      <c r="L36" s="15"/>
+      <c r="M36" s="15">
         <v>0.3</v>
       </c>
     </row>
@@ -1944,17 +1941,17 @@
       <c r="H37" s="3">
         <v>94.4</v>
       </c>
-      <c r="I37" s="21" t="s">
+      <c r="I37" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J37" s="21">
+      <c r="J37" s="15">
         <v>9.4</v>
       </c>
-      <c r="K37" s="21"/>
-      <c r="L37" s="21">
+      <c r="K37" s="15"/>
+      <c r="L37" s="15">
         <v>5.6</v>
       </c>
-      <c r="M37" s="21">
+      <c r="M37" s="15">
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
@@ -1981,17 +1978,17 @@
       <c r="H38" s="3">
         <v>464.04</v>
       </c>
-      <c r="I38" s="21" t="s">
+      <c r="I38" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J38" s="21">
+      <c r="J38" s="15">
         <v>8.9</v>
       </c>
-      <c r="K38" s="21"/>
-      <c r="L38" s="21">
+      <c r="K38" s="15"/>
+      <c r="L38" s="15">
         <v>7.73</v>
       </c>
-      <c r="M38" s="21">
+      <c r="M38" s="15">
         <v>1.1000000000000001</v>
       </c>
     </row>
@@ -2016,15 +2013,15 @@
       <c r="H39" s="3">
         <v>847.09</v>
       </c>
-      <c r="I39" s="21" t="s">
+      <c r="I39" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J39" s="21"/>
-      <c r="K39" s="21"/>
-      <c r="L39" s="21">
+      <c r="J39" s="15"/>
+      <c r="K39" s="15"/>
+      <c r="L39" s="15">
         <v>5.3</v>
       </c>
-      <c r="M39" s="21"/>
+      <c r="M39" s="15"/>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
@@ -2051,17 +2048,17 @@
       <c r="H40" s="3">
         <v>744.89</v>
       </c>
-      <c r="I40" s="21" t="s">
+      <c r="I40" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J40" s="21">
+      <c r="J40" s="15">
         <v>11.6</v>
       </c>
-      <c r="K40" s="21"/>
-      <c r="L40" s="21">
+      <c r="K40" s="15"/>
+      <c r="L40" s="15">
         <v>2.9</v>
       </c>
-      <c r="M40" s="21">
+      <c r="M40" s="15">
         <v>2.7</v>
       </c>
     </row>
@@ -2088,15 +2085,15 @@
       <c r="H41" s="3">
         <v>1249.8599999999999</v>
       </c>
-      <c r="I41" s="21"/>
-      <c r="J41" s="21">
+      <c r="I41" s="15"/>
+      <c r="J41" s="15">
         <v>19.2</v>
       </c>
-      <c r="K41" s="21">
+      <c r="K41" s="15">
         <v>14.6</v>
       </c>
-      <c r="L41" s="21"/>
-      <c r="M41" s="21"/>
+      <c r="L41" s="15"/>
+      <c r="M41" s="15"/>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
@@ -2123,11 +2120,11 @@
       <c r="H42" s="3">
         <v>11.05</v>
       </c>
-      <c r="I42" s="21"/>
-      <c r="J42" s="21"/>
-      <c r="K42" s="21"/>
-      <c r="L42" s="21"/>
-      <c r="M42" s="21"/>
+      <c r="I42" s="15"/>
+      <c r="J42" s="15"/>
+      <c r="K42" s="15"/>
+      <c r="L42" s="15"/>
+      <c r="M42" s="15"/>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
@@ -2150,17 +2147,17 @@
       <c r="H43" s="3">
         <v>2500</v>
       </c>
-      <c r="I43" s="21" t="s">
+      <c r="I43" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J43" s="21"/>
-      <c r="K43" s="21">
+      <c r="J43" s="15"/>
+      <c r="K43" s="15">
         <v>21.4</v>
       </c>
-      <c r="L43" s="21">
+      <c r="L43" s="15">
         <v>22.5</v>
       </c>
-      <c r="M43" s="21">
+      <c r="M43" s="15">
         <v>9.1999999999999993</v>
       </c>
     </row>
@@ -2187,17 +2184,17 @@
       <c r="H44" s="3">
         <v>12.66</v>
       </c>
-      <c r="I44" s="21" t="s">
+      <c r="I44" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J44" s="21"/>
-      <c r="K44" s="21">
+      <c r="J44" s="15"/>
+      <c r="K44" s="15">
         <v>22.3</v>
       </c>
-      <c r="L44" s="21">
+      <c r="L44" s="15">
         <v>23.6</v>
       </c>
-      <c r="M44" s="21">
+      <c r="M44" s="15">
         <v>8.3000000000000007</v>
       </c>
     </row>
@@ -2224,17 +2221,17 @@
       <c r="H45" s="3">
         <v>14.26</v>
       </c>
-      <c r="I45" s="21"/>
-      <c r="J45" s="21">
+      <c r="I45" s="15"/>
+      <c r="J45" s="15">
         <v>12.5</v>
       </c>
-      <c r="K45" s="21">
+      <c r="K45" s="15">
         <v>20</v>
       </c>
-      <c r="L45" s="21">
+      <c r="L45" s="15">
         <v>19.3</v>
       </c>
-      <c r="M45" s="21">
+      <c r="M45" s="15">
         <v>5.4</v>
       </c>
     </row>
@@ -2261,15 +2258,15 @@
       <c r="H46" s="3">
         <v>11.02</v>
       </c>
-      <c r="I46" s="21"/>
-      <c r="J46" s="21"/>
-      <c r="K46" s="21">
+      <c r="I46" s="15"/>
+      <c r="J46" s="15"/>
+      <c r="K46" s="15">
         <v>4.3</v>
       </c>
-      <c r="L46" s="21">
+      <c r="L46" s="15">
         <v>9.3222000000000005</v>
       </c>
-      <c r="M46" s="21"/>
+      <c r="M46" s="15"/>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
@@ -2294,19 +2291,19 @@
       <c r="H47" s="3">
         <v>12.5</v>
       </c>
-      <c r="I47" s="21" t="s">
+      <c r="I47" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J47" s="21">
+      <c r="J47" s="15">
         <v>8.1999999999999993</v>
       </c>
-      <c r="K47" s="21">
+      <c r="K47" s="15">
         <v>7.3</v>
       </c>
-      <c r="L47" s="21">
+      <c r="L47" s="15">
         <v>6.3</v>
       </c>
-      <c r="M47" s="21">
+      <c r="M47" s="15">
         <v>0.2</v>
       </c>
     </row>
@@ -2333,17 +2330,17 @@
       <c r="H48" s="3">
         <v>48.65</v>
       </c>
-      <c r="I48" s="21"/>
-      <c r="J48" s="21">
+      <c r="I48" s="15"/>
+      <c r="J48" s="15">
         <v>9.1199999999999992</v>
       </c>
-      <c r="K48" s="21">
+      <c r="K48" s="15">
         <v>11.9</v>
       </c>
-      <c r="L48" s="21">
+      <c r="L48" s="15">
         <v>4.3</v>
       </c>
-      <c r="M48" s="21"/>
+      <c r="M48" s="15"/>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
@@ -2370,15 +2367,15 @@
       <c r="H49" s="3">
         <v>47.96</v>
       </c>
-      <c r="I49" s="21" t="s">
+      <c r="I49" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J49" s="21">
+      <c r="J49" s="15">
         <v>16.8</v>
       </c>
-      <c r="K49" s="21"/>
-      <c r="L49" s="21"/>
-      <c r="M49" s="21"/>
+      <c r="K49" s="15"/>
+      <c r="L49" s="15"/>
+      <c r="M49" s="15"/>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
@@ -2403,15 +2400,15 @@
       <c r="H50" s="3">
         <v>9.92</v>
       </c>
-      <c r="I50" s="21" t="s">
+      <c r="I50" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J50" s="21">
+      <c r="J50" s="15">
         <v>21</v>
       </c>
-      <c r="K50" s="21"/>
-      <c r="L50" s="21"/>
-      <c r="M50" s="21">
+      <c r="K50" s="15"/>
+      <c r="L50" s="15"/>
+      <c r="M50" s="15">
         <v>10.199999999999999</v>
       </c>
     </row>
@@ -2438,11 +2435,11 @@
       <c r="H51" s="3">
         <v>13.4</v>
       </c>
-      <c r="I51" s="21"/>
-      <c r="J51" s="21"/>
-      <c r="K51" s="21"/>
-      <c r="L51" s="21"/>
-      <c r="M51" s="21"/>
+      <c r="I51" s="15"/>
+      <c r="J51" s="15"/>
+      <c r="K51" s="15"/>
+      <c r="L51" s="15"/>
+      <c r="M51" s="15"/>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A52" s="2">
@@ -2467,15 +2464,15 @@
       <c r="H52" s="3">
         <v>10.210000000000001</v>
       </c>
-      <c r="I52" s="21"/>
-      <c r="J52" s="21"/>
-      <c r="K52" s="21">
+      <c r="I52" s="15"/>
+      <c r="J52" s="15"/>
+      <c r="K52" s="15">
         <v>19.399999999999999</v>
       </c>
-      <c r="L52" s="21">
+      <c r="L52" s="15">
         <v>5.34</v>
       </c>
-      <c r="M52" s="21"/>
+      <c r="M52" s="15"/>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A53" s="2">
@@ -2500,11 +2497,11 @@
       <c r="H53" s="3">
         <v>12.96</v>
       </c>
-      <c r="I53" s="21"/>
-      <c r="J53" s="21"/>
-      <c r="K53" s="21"/>
-      <c r="L53" s="21"/>
-      <c r="M53" s="21"/>
+      <c r="I53" s="15"/>
+      <c r="J53" s="15"/>
+      <c r="K53" s="15"/>
+      <c r="L53" s="15"/>
+      <c r="M53" s="15"/>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A54" s="2">
@@ -2529,19 +2526,19 @@
       <c r="H54" s="3">
         <v>751.95</v>
       </c>
-      <c r="I54" s="21" t="s">
+      <c r="I54" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J54" s="21">
+      <c r="J54" s="15">
         <v>18.2</v>
       </c>
-      <c r="K54" s="21">
+      <c r="K54" s="15">
         <v>16.8</v>
       </c>
-      <c r="L54" s="21">
+      <c r="L54" s="15">
         <v>4.9000000000000004</v>
       </c>
-      <c r="M54" s="21">
+      <c r="M54" s="15">
         <v>0.5</v>
       </c>
     </row>
@@ -2568,13 +2565,13 @@
       <c r="H55" s="3">
         <v>23.58</v>
       </c>
-      <c r="I55" s="21"/>
-      <c r="J55" s="21"/>
-      <c r="K55" s="21"/>
-      <c r="L55" s="21">
+      <c r="I55" s="15"/>
+      <c r="J55" s="15"/>
+      <c r="K55" s="15"/>
+      <c r="L55" s="15">
         <v>6.9</v>
       </c>
-      <c r="M55" s="21"/>
+      <c r="M55" s="15"/>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A56" s="2">
@@ -2599,19 +2596,19 @@
       <c r="H56" s="3">
         <v>11.52</v>
       </c>
-      <c r="I56" s="21" t="s">
+      <c r="I56" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J56" s="21">
+      <c r="J56" s="15">
         <v>11.7</v>
       </c>
-      <c r="K56" s="21">
+      <c r="K56" s="15">
         <v>23.7</v>
       </c>
-      <c r="L56" s="21">
+      <c r="L56" s="15">
         <v>3.7</v>
       </c>
-      <c r="M56" s="21">
+      <c r="M56" s="15">
         <v>1.2</v>
       </c>
     </row>
@@ -2640,19 +2637,19 @@
       <c r="H57" s="3">
         <v>53.42</v>
       </c>
-      <c r="I57" s="21" t="s">
+      <c r="I57" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J57" s="21">
+      <c r="J57" s="15">
         <v>10.199999999999999</v>
       </c>
-      <c r="K57" s="21">
+      <c r="K57" s="15">
         <v>20.399999999999999</v>
       </c>
-      <c r="L57" s="21">
+      <c r="L57" s="15">
         <v>11.5</v>
       </c>
-      <c r="M57" s="21">
+      <c r="M57" s="15">
         <v>1.08</v>
       </c>
     </row>
@@ -2681,11 +2678,11 @@
       <c r="H58" s="3">
         <v>38.729999999999997</v>
       </c>
-      <c r="I58" s="21"/>
-      <c r="J58" s="21"/>
-      <c r="K58" s="21"/>
-      <c r="L58" s="21"/>
-      <c r="M58" s="21"/>
+      <c r="I58" s="15"/>
+      <c r="J58" s="15"/>
+      <c r="K58" s="15"/>
+      <c r="L58" s="15"/>
+      <c r="M58" s="15"/>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A59" s="2">
@@ -2712,13 +2709,13 @@
       <c r="H59" s="3">
         <v>24.36</v>
       </c>
-      <c r="I59" s="21"/>
-      <c r="J59" s="21">
+      <c r="I59" s="15"/>
+      <c r="J59" s="15">
         <v>17.5</v>
       </c>
-      <c r="K59" s="21"/>
-      <c r="L59" s="21"/>
-      <c r="M59" s="21"/>
+      <c r="K59" s="15"/>
+      <c r="L59" s="15"/>
+      <c r="M59" s="15"/>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A60" s="2">
@@ -2745,17 +2742,17 @@
       <c r="H60" s="3">
         <v>33.049999999999997</v>
       </c>
-      <c r="I60" s="21" t="s">
+      <c r="I60" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J60" s="21"/>
-      <c r="K60" s="21">
+      <c r="J60" s="15"/>
+      <c r="K60" s="15">
         <v>12.9</v>
       </c>
-      <c r="L60" s="21">
+      <c r="L60" s="15">
         <v>5.3</v>
       </c>
-      <c r="M60" s="21">
+      <c r="M60" s="15">
         <v>0.6</v>
       </c>
     </row>
@@ -2780,11 +2777,11 @@
       <c r="H61" s="3">
         <v>710.2</v>
       </c>
-      <c r="I61" s="21"/>
-      <c r="J61" s="21"/>
-      <c r="K61" s="21"/>
-      <c r="L61" s="21"/>
-      <c r="M61" s="21"/>
+      <c r="I61" s="15"/>
+      <c r="J61" s="15"/>
+      <c r="K61" s="15"/>
+      <c r="L61" s="15"/>
+      <c r="M61" s="15"/>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A62" s="2">
@@ -2809,11 +2806,11 @@
       <c r="H62" s="3">
         <v>406.72</v>
       </c>
-      <c r="I62" s="21"/>
-      <c r="J62" s="21"/>
-      <c r="K62" s="21"/>
-      <c r="L62" s="21"/>
-      <c r="M62" s="21"/>
+      <c r="I62" s="15"/>
+      <c r="J62" s="15"/>
+      <c r="K62" s="15"/>
+      <c r="L62" s="15"/>
+      <c r="M62" s="15"/>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A63" s="2">
@@ -2838,19 +2835,19 @@
       <c r="H63" s="3">
         <v>27.69</v>
       </c>
-      <c r="I63" s="21" t="s">
+      <c r="I63" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J63" s="21">
+      <c r="J63" s="15">
         <v>8.8000000000000007</v>
       </c>
-      <c r="K63" s="21">
+      <c r="K63" s="15">
         <v>11.9</v>
       </c>
-      <c r="L63" s="21">
+      <c r="L63" s="15">
         <v>6.3</v>
       </c>
-      <c r="M63" s="21">
+      <c r="M63" s="15">
         <v>1.2</v>
       </c>
     </row>
@@ -2879,19 +2876,19 @@
       <c r="H64" s="3">
         <v>34.549999999999997</v>
       </c>
-      <c r="I64" s="21" t="s">
+      <c r="I64" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J64" s="21">
+      <c r="J64" s="15">
         <v>9.3000000000000007</v>
       </c>
-      <c r="K64" s="21">
+      <c r="K64" s="15">
         <v>13.2</v>
       </c>
-      <c r="L64" s="21">
+      <c r="L64" s="15">
         <v>7.3</v>
       </c>
-      <c r="M64" s="21">
+      <c r="M64" s="15">
         <v>0.91</v>
       </c>
     </row>
@@ -2920,11 +2917,11 @@
       <c r="H65" s="3">
         <v>29.24</v>
       </c>
-      <c r="I65" s="21"/>
-      <c r="J65" s="21"/>
-      <c r="K65" s="21"/>
-      <c r="L65" s="21"/>
-      <c r="M65" s="21"/>
+      <c r="I65" s="15"/>
+      <c r="J65" s="15"/>
+      <c r="K65" s="15"/>
+      <c r="L65" s="15"/>
+      <c r="M65" s="15"/>
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A66" s="2">
@@ -2949,11 +2946,11 @@
       <c r="H66" s="3">
         <v>482.11</v>
       </c>
-      <c r="I66" s="21"/>
-      <c r="J66" s="21"/>
-      <c r="K66" s="21"/>
-      <c r="L66" s="21"/>
-      <c r="M66" s="21"/>
+      <c r="I66" s="15"/>
+      <c r="J66" s="15"/>
+      <c r="K66" s="15"/>
+      <c r="L66" s="15"/>
+      <c r="M66" s="15"/>
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A67" s="2">
@@ -2978,19 +2975,19 @@
       <c r="H67" s="3">
         <v>44.23</v>
       </c>
-      <c r="I67" s="21" t="s">
+      <c r="I67" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J67" s="21">
+      <c r="J67" s="15">
         <v>14.4</v>
       </c>
-      <c r="K67" s="21">
+      <c r="K67" s="15">
         <v>19.399999999999999</v>
       </c>
-      <c r="L67" s="21">
+      <c r="L67" s="15">
         <v>3.8</v>
       </c>
-      <c r="M67" s="21">
+      <c r="M67" s="15">
         <v>0.3</v>
       </c>
     </row>
@@ -3017,11 +3014,11 @@
       <c r="H68" s="3">
         <v>229.3</v>
       </c>
-      <c r="I68" s="21"/>
-      <c r="J68" s="21"/>
-      <c r="K68" s="21"/>
-      <c r="L68" s="21"/>
-      <c r="M68" s="21"/>
+      <c r="I68" s="15"/>
+      <c r="J68" s="15"/>
+      <c r="K68" s="15"/>
+      <c r="L68" s="15"/>
+      <c r="M68" s="15"/>
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A69" s="2">
@@ -3046,11 +3043,11 @@
       <c r="H69" s="3">
         <v>4.7699999999999996</v>
       </c>
-      <c r="I69" s="21"/>
-      <c r="J69" s="21"/>
-      <c r="K69" s="21"/>
-      <c r="L69" s="21"/>
-      <c r="M69" s="21"/>
+      <c r="I69" s="15"/>
+      <c r="J69" s="15"/>
+      <c r="K69" s="15"/>
+      <c r="L69" s="15"/>
+      <c r="M69" s="15"/>
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A70" s="2">
@@ -3075,19 +3072,19 @@
       <c r="H70" s="3">
         <v>96.33</v>
       </c>
-      <c r="I70" s="21" t="s">
+      <c r="I70" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J70" s="21">
+      <c r="J70" s="15">
         <v>29.6</v>
       </c>
-      <c r="K70" s="21">
+      <c r="K70" s="15">
         <v>31.4</v>
       </c>
-      <c r="L70" s="21">
+      <c r="L70" s="15">
         <v>29.2</v>
       </c>
-      <c r="M70" s="21">
+      <c r="M70" s="15">
         <v>11.2</v>
       </c>
     </row>
@@ -3114,19 +3111,19 @@
       <c r="H71" s="3">
         <v>71.89</v>
       </c>
-      <c r="I71" s="21" t="s">
+      <c r="I71" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J71" s="21">
+      <c r="J71" s="15">
         <v>25.8</v>
       </c>
-      <c r="K71" s="21">
+      <c r="K71" s="15">
         <v>29.4</v>
       </c>
-      <c r="L71" s="21">
+      <c r="L71" s="15">
         <v>25.4</v>
       </c>
-      <c r="M71" s="21">
+      <c r="M71" s="15">
         <v>9.3000000000000007</v>
       </c>
     </row>
@@ -3153,19 +3150,19 @@
       <c r="H72" s="3">
         <v>60.39</v>
       </c>
-      <c r="I72" s="21" t="s">
+      <c r="I72" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J72" s="21">
+      <c r="J72" s="15">
         <v>29.2</v>
       </c>
-      <c r="K72" s="21">
+      <c r="K72" s="15">
         <v>22.7</v>
       </c>
-      <c r="L72" s="21">
+      <c r="L72" s="15">
         <v>23.3</v>
       </c>
-      <c r="M72" s="21">
+      <c r="M72" s="15">
         <v>5.4</v>
       </c>
     </row>
@@ -3192,19 +3189,19 @@
       <c r="H73" s="3">
         <v>35.17</v>
       </c>
-      <c r="I73" s="21" t="s">
+      <c r="I73" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J73" s="21">
+      <c r="J73" s="15">
         <v>9.4</v>
       </c>
-      <c r="K73" s="21">
+      <c r="K73" s="15">
         <v>11.3</v>
       </c>
-      <c r="L73" s="21">
+      <c r="L73" s="15">
         <v>11.1</v>
       </c>
-      <c r="M73" s="21">
+      <c r="M73" s="15">
         <v>2.1</v>
       </c>
     </row>
@@ -3233,11 +3230,11 @@
       <c r="H74" s="3">
         <v>24.48</v>
       </c>
-      <c r="I74" s="21"/>
-      <c r="J74" s="21"/>
-      <c r="K74" s="21"/>
-      <c r="L74" s="21"/>
-      <c r="M74" s="21"/>
+      <c r="I74" s="15"/>
+      <c r="J74" s="15"/>
+      <c r="K74" s="15"/>
+      <c r="L74" s="15"/>
+      <c r="M74" s="15"/>
     </row>
     <row r="75" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A75" s="3" t="s">
@@ -3262,13 +3259,13 @@
       <c r="H75" s="3">
         <v>19.079999999999998</v>
       </c>
-      <c r="I75" s="21" t="s">
+      <c r="I75" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J75" s="21"/>
-      <c r="K75" s="21"/>
-      <c r="L75" s="21"/>
-      <c r="M75" s="21"/>
+      <c r="J75" s="15"/>
+      <c r="K75" s="15"/>
+      <c r="L75" s="15"/>
+      <c r="M75" s="15"/>
     </row>
     <row r="76" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A76" s="3" t="s">
@@ -3293,19 +3290,19 @@
       <c r="H76" s="3">
         <v>17.18</v>
       </c>
-      <c r="I76" s="21" t="s">
+      <c r="I76" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J76" s="21">
+      <c r="J76" s="15">
         <v>4.8</v>
       </c>
-      <c r="K76" s="21">
+      <c r="K76" s="15">
         <v>22.9</v>
       </c>
-      <c r="L76" s="21">
+      <c r="L76" s="15">
         <v>7.3</v>
       </c>
-      <c r="M76" s="21">
+      <c r="M76" s="15">
         <v>0.2</v>
       </c>
     </row>
@@ -3332,11 +3329,11 @@
       <c r="H77" s="3">
         <v>15.17</v>
       </c>
-      <c r="I77" s="21"/>
-      <c r="J77" s="21"/>
-      <c r="K77" s="21"/>
-      <c r="L77" s="21"/>
-      <c r="M77" s="21"/>
+      <c r="I77" s="15"/>
+      <c r="J77" s="15"/>
+      <c r="K77" s="15"/>
+      <c r="L77" s="15"/>
+      <c r="M77" s="15"/>
     </row>
     <row r="78" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A78" s="3" t="s">
@@ -3361,17 +3358,17 @@
       <c r="H78" s="3">
         <v>22.3</v>
       </c>
-      <c r="I78" s="21" t="s">
+      <c r="I78" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J78" s="21">
+      <c r="J78" s="15">
         <v>22.7</v>
       </c>
-      <c r="K78" s="21"/>
-      <c r="L78" s="21">
+      <c r="K78" s="15"/>
+      <c r="L78" s="15">
         <v>22.2</v>
       </c>
-      <c r="M78" s="21">
+      <c r="M78" s="15">
         <v>5.8</v>
       </c>
     </row>
@@ -3398,19 +3395,19 @@
       <c r="H79" s="3">
         <v>113.3</v>
       </c>
-      <c r="I79" s="21" t="s">
+      <c r="I79" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J79" s="21">
+      <c r="J79" s="15">
         <v>14.7</v>
       </c>
-      <c r="K79" s="21">
+      <c r="K79" s="15">
         <v>19.8</v>
       </c>
-      <c r="L79" s="21">
+      <c r="L79" s="15">
         <v>6.8</v>
       </c>
-      <c r="M79" s="21">
+      <c r="M79" s="15">
         <v>1.1000000000000001</v>
       </c>
     </row>
@@ -3437,19 +3434,19 @@
       <c r="H80" s="3">
         <v>57.01</v>
       </c>
-      <c r="I80" s="21" t="s">
+      <c r="I80" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J80" s="21">
+      <c r="J80" s="15">
         <v>18.5</v>
       </c>
-      <c r="K80" s="21">
+      <c r="K80" s="15">
         <v>24.7</v>
       </c>
-      <c r="L80" s="21">
+      <c r="L80" s="15">
         <v>11.4</v>
       </c>
-      <c r="M80" s="21">
+      <c r="M80" s="15">
         <v>7.1</v>
       </c>
     </row>
@@ -3476,11 +3473,11 @@
       <c r="H81" s="3">
         <v>360.3</v>
       </c>
-      <c r="I81" s="21"/>
-      <c r="J81" s="21"/>
-      <c r="K81" s="21"/>
-      <c r="L81" s="21"/>
-      <c r="M81" s="21"/>
+      <c r="I81" s="15"/>
+      <c r="J81" s="15"/>
+      <c r="K81" s="15"/>
+      <c r="L81" s="15"/>
+      <c r="M81" s="15"/>
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A82" s="3" t="s">
@@ -3505,11 +3502,11 @@
       <c r="H82" s="3">
         <v>126.13</v>
       </c>
-      <c r="I82" s="21"/>
-      <c r="J82" s="21"/>
-      <c r="K82" s="21"/>
-      <c r="L82" s="21"/>
-      <c r="M82" s="21"/>
+      <c r="I82" s="15"/>
+      <c r="J82" s="15"/>
+      <c r="K82" s="15"/>
+      <c r="L82" s="15"/>
+      <c r="M82" s="15"/>
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A83" s="3" t="s">
@@ -3534,19 +3531,19 @@
       <c r="H83" s="3">
         <v>12.32</v>
       </c>
-      <c r="I83" s="21" t="s">
+      <c r="I83" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J83" s="21">
+      <c r="J83" s="15">
         <v>41.3</v>
       </c>
-      <c r="K83" s="21">
+      <c r="K83" s="15">
         <v>26.5</v>
       </c>
-      <c r="L83" s="21">
+      <c r="L83" s="15">
         <v>19.600000000000001</v>
       </c>
-      <c r="M83" s="21">
+      <c r="M83" s="15">
         <v>7.6</v>
       </c>
     </row>
@@ -3573,19 +3570,19 @@
       <c r="H84" s="3">
         <v>30.96</v>
       </c>
-      <c r="I84" s="21" t="s">
+      <c r="I84" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J84" s="21">
+      <c r="J84" s="15">
         <v>33.799999999999997</v>
       </c>
-      <c r="K84" s="21">
+      <c r="K84" s="15">
         <v>19.7</v>
       </c>
-      <c r="L84" s="21">
+      <c r="L84" s="15">
         <v>21.9</v>
       </c>
-      <c r="M84" s="21">
+      <c r="M84" s="15">
         <v>9.1999999999999993</v>
       </c>
     </row>
@@ -3612,11 +3609,11 @@
       <c r="H85" s="3">
         <v>19.7</v>
       </c>
-      <c r="I85" s="21"/>
-      <c r="J85" s="21"/>
-      <c r="K85" s="21"/>
-      <c r="L85" s="21"/>
-      <c r="M85" s="21"/>
+      <c r="I85" s="15"/>
+      <c r="J85" s="15"/>
+      <c r="K85" s="15"/>
+      <c r="L85" s="15"/>
+      <c r="M85" s="15"/>
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A86" s="3" t="s">
@@ -3641,11 +3638,11 @@
       <c r="H86" s="3">
         <v>19.23</v>
       </c>
-      <c r="I86" s="21"/>
-      <c r="J86" s="21"/>
-      <c r="K86" s="21"/>
-      <c r="L86" s="21"/>
-      <c r="M86" s="21"/>
+      <c r="I86" s="15"/>
+      <c r="J86" s="15"/>
+      <c r="K86" s="15"/>
+      <c r="L86" s="15"/>
+      <c r="M86" s="15"/>
     </row>
     <row r="87" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A87" s="3" t="s">
@@ -3670,13 +3667,13 @@
       <c r="H87" s="3">
         <v>301.7</v>
       </c>
-      <c r="I87" s="21"/>
-      <c r="J87" s="21"/>
-      <c r="K87" s="21"/>
-      <c r="L87" s="21">
+      <c r="I87" s="15"/>
+      <c r="J87" s="15"/>
+      <c r="K87" s="15"/>
+      <c r="L87" s="15">
         <v>12.2</v>
       </c>
-      <c r="M87" s="21">
+      <c r="M87" s="15">
         <v>8.3000000000000007</v>
       </c>
     </row>
@@ -3705,15 +3702,15 @@
       <c r="H88" s="3">
         <v>39.39</v>
       </c>
-      <c r="I88" s="21"/>
-      <c r="J88" s="21"/>
-      <c r="K88" s="21">
+      <c r="I88" s="15"/>
+      <c r="J88" s="15"/>
+      <c r="K88" s="15">
         <v>16.600000000000001</v>
       </c>
-      <c r="L88" s="21">
+      <c r="L88" s="15">
         <v>17.7</v>
       </c>
-      <c r="M88" s="21">
+      <c r="M88" s="15">
         <v>7.7</v>
       </c>
     </row>
@@ -3742,11 +3739,11 @@
       <c r="H89" s="3">
         <v>38.46</v>
       </c>
-      <c r="I89" s="21"/>
-      <c r="J89" s="21"/>
-      <c r="K89" s="21"/>
-      <c r="L89" s="21"/>
-      <c r="M89" s="21"/>
+      <c r="I89" s="15"/>
+      <c r="J89" s="15"/>
+      <c r="K89" s="15"/>
+      <c r="L89" s="15"/>
+      <c r="M89" s="15"/>
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A90" s="3" t="s">
@@ -3771,11 +3768,11 @@
       <c r="H90" s="3">
         <v>14.69</v>
       </c>
-      <c r="I90" s="21"/>
-      <c r="J90" s="21"/>
-      <c r="K90" s="21"/>
-      <c r="L90" s="21"/>
-      <c r="M90" s="21"/>
+      <c r="I90" s="15"/>
+      <c r="J90" s="15"/>
+      <c r="K90" s="15"/>
+      <c r="L90" s="15"/>
+      <c r="M90" s="15"/>
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A91" s="3" t="s">
@@ -3800,11 +3797,11 @@
       <c r="H91" s="3">
         <v>14.36</v>
       </c>
-      <c r="I91" s="21"/>
-      <c r="J91" s="21"/>
-      <c r="K91" s="21"/>
-      <c r="L91" s="21"/>
-      <c r="M91" s="21"/>
+      <c r="I91" s="15"/>
+      <c r="J91" s="15"/>
+      <c r="K91" s="15"/>
+      <c r="L91" s="15"/>
+      <c r="M91" s="15"/>
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A92" s="3" t="s">
@@ -3831,19 +3828,19 @@
       <c r="H92" s="3">
         <v>15.81</v>
       </c>
-      <c r="I92" s="21" t="s">
+      <c r="I92" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J92" s="21">
+      <c r="J92" s="15">
         <v>14.7</v>
       </c>
-      <c r="K92" s="21">
+      <c r="K92" s="15">
         <v>11.8</v>
       </c>
-      <c r="L92" s="21">
+      <c r="L92" s="15">
         <v>8.8800000000000008</v>
       </c>
-      <c r="M92" s="21">
+      <c r="M92" s="15">
         <v>1.3</v>
       </c>
     </row>
@@ -3872,11 +3869,11 @@
       <c r="H93" s="3">
         <v>31.64</v>
       </c>
-      <c r="I93" s="21"/>
-      <c r="J93" s="21"/>
-      <c r="K93" s="21"/>
-      <c r="L93" s="21"/>
-      <c r="M93" s="21"/>
+      <c r="I93" s="15"/>
+      <c r="J93" s="15"/>
+      <c r="K93" s="15"/>
+      <c r="L93" s="15"/>
+      <c r="M93" s="15"/>
     </row>
     <row r="94" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A94" s="3" t="s">
@@ -3903,15 +3900,15 @@
       <c r="H94" s="3">
         <v>33.89</v>
       </c>
-      <c r="I94" s="21"/>
-      <c r="J94" s="21"/>
-      <c r="K94" s="21">
+      <c r="I94" s="15"/>
+      <c r="J94" s="15"/>
+      <c r="K94" s="15">
         <v>23.6</v>
       </c>
-      <c r="L94" s="21">
+      <c r="L94" s="15">
         <v>9.1999999999999993</v>
       </c>
-      <c r="M94" s="21">
+      <c r="M94" s="15">
         <v>2.2000000000000002</v>
       </c>
     </row>
@@ -3938,11 +3935,11 @@
       <c r="H95" s="3">
         <v>19.3</v>
       </c>
-      <c r="I95" s="21"/>
-      <c r="J95" s="21"/>
-      <c r="K95" s="21"/>
-      <c r="L95" s="21"/>
-      <c r="M95" s="21"/>
+      <c r="I95" s="15"/>
+      <c r="J95" s="15"/>
+      <c r="K95" s="15"/>
+      <c r="L95" s="15"/>
+      <c r="M95" s="15"/>
     </row>
     <row r="96" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A96" s="3" t="s">
@@ -3967,11 +3964,11 @@
       <c r="H96" s="3">
         <v>20.32</v>
       </c>
-      <c r="I96" s="21"/>
-      <c r="J96" s="21"/>
-      <c r="K96" s="21"/>
-      <c r="L96" s="21"/>
-      <c r="M96" s="21"/>
+      <c r="I96" s="15"/>
+      <c r="J96" s="15"/>
+      <c r="K96" s="15"/>
+      <c r="L96" s="15"/>
+      <c r="M96" s="15"/>
     </row>
     <row r="97" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A97" s="3" t="s">
@@ -3996,19 +3993,19 @@
       <c r="H97" s="3">
         <v>210.42</v>
       </c>
-      <c r="I97" s="21" t="s">
+      <c r="I97" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J97" s="21">
+      <c r="J97" s="15">
         <v>17.399999999999999</v>
       </c>
-      <c r="K97" s="21">
+      <c r="K97" s="15">
         <v>21.7</v>
       </c>
-      <c r="L97" s="21">
+      <c r="L97" s="15">
         <v>7.2</v>
       </c>
-      <c r="M97" s="21">
+      <c r="M97" s="15">
         <v>1.2</v>
       </c>
     </row>
@@ -4033,11 +4030,11 @@
       <c r="H98" s="3">
         <v>427</v>
       </c>
-      <c r="I98" s="21"/>
-      <c r="J98" s="21"/>
-      <c r="K98" s="21"/>
-      <c r="L98" s="21"/>
-      <c r="M98" s="21"/>
+      <c r="I98" s="15"/>
+      <c r="J98" s="15"/>
+      <c r="K98" s="15"/>
+      <c r="L98" s="15"/>
+      <c r="M98" s="15"/>
     </row>
     <row r="99" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A99" s="3" t="s">
@@ -4062,11 +4059,11 @@
       <c r="H99" s="3">
         <v>21.23</v>
       </c>
-      <c r="I99" s="21"/>
-      <c r="J99" s="21"/>
-      <c r="K99" s="21"/>
-      <c r="L99" s="21"/>
-      <c r="M99" s="21"/>
+      <c r="I99" s="15"/>
+      <c r="J99" s="15"/>
+      <c r="K99" s="15"/>
+      <c r="L99" s="15"/>
+      <c r="M99" s="15"/>
     </row>
     <row r="100" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A100" s="3" t="s">
@@ -4093,19 +4090,19 @@
       <c r="H100" s="3">
         <v>13.17</v>
       </c>
-      <c r="I100" s="21" t="s">
+      <c r="I100" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J100" s="21">
+      <c r="J100" s="15">
         <v>23.5</v>
       </c>
-      <c r="K100" s="21">
+      <c r="K100" s="15">
         <v>25.8</v>
       </c>
-      <c r="L100" s="21">
+      <c r="L100" s="15">
         <v>15.8</v>
       </c>
-      <c r="M100" s="21">
+      <c r="M100" s="15">
         <v>4.7</v>
       </c>
     </row>
@@ -4134,13 +4131,13 @@
       <c r="H101" s="3">
         <v>8.7100000000000009</v>
       </c>
-      <c r="I101" s="21"/>
-      <c r="J101" s="21">
+      <c r="I101" s="15"/>
+      <c r="J101" s="15">
         <v>25.3</v>
       </c>
-      <c r="K101" s="21"/>
-      <c r="L101" s="21"/>
-      <c r="M101" s="21"/>
+      <c r="K101" s="15"/>
+      <c r="L101" s="15"/>
+      <c r="M101" s="15"/>
     </row>
     <row r="102" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A102" s="3" t="s">
@@ -4165,11 +4162,11 @@
       <c r="H102" s="3">
         <v>69.61</v>
       </c>
-      <c r="I102" s="21"/>
-      <c r="J102" s="21"/>
-      <c r="K102" s="21"/>
-      <c r="L102" s="21"/>
-      <c r="M102" s="21"/>
+      <c r="I102" s="15"/>
+      <c r="J102" s="15"/>
+      <c r="K102" s="15"/>
+      <c r="L102" s="15"/>
+      <c r="M102" s="15"/>
     </row>
     <row r="103" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A103" s="3" t="s">
@@ -4194,13 +4191,13 @@
       <c r="H103" s="3">
         <v>226.61</v>
       </c>
-      <c r="I103" s="21" t="s">
+      <c r="I103" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J103" s="21"/>
-      <c r="K103" s="21"/>
-      <c r="L103" s="21"/>
-      <c r="M103" s="21"/>
+      <c r="J103" s="15"/>
+      <c r="K103" s="15"/>
+      <c r="L103" s="15"/>
+      <c r="M103" s="15"/>
     </row>
     <row r="104" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A104" s="3" t="s">
@@ -4225,19 +4222,19 @@
       <c r="H104" s="3">
         <v>336.03</v>
       </c>
-      <c r="I104" s="21" t="s">
+      <c r="I104" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J104" s="21">
+      <c r="J104" s="15">
         <v>21.4</v>
       </c>
-      <c r="K104" s="21">
+      <c r="K104" s="15">
         <v>19.399999999999999</v>
       </c>
-      <c r="L104" s="21">
+      <c r="L104" s="15">
         <v>11.1</v>
       </c>
-      <c r="M104" s="21">
+      <c r="M104" s="15">
         <v>1.3</v>
       </c>
     </row>
@@ -4264,19 +4261,19 @@
       <c r="H105" s="3">
         <v>101.2</v>
       </c>
-      <c r="I105" s="21" t="s">
+      <c r="I105" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J105" s="21">
+      <c r="J105" s="15">
         <v>25.7</v>
       </c>
-      <c r="K105" s="21">
+      <c r="K105" s="15">
         <v>23.1</v>
       </c>
-      <c r="L105" s="21">
+      <c r="L105" s="15">
         <v>21.8</v>
       </c>
-      <c r="M105" s="21">
+      <c r="M105" s="15">
         <v>12.7</v>
       </c>
     </row>
@@ -4303,11 +4300,11 @@
       <c r="H106" s="3">
         <v>14.5</v>
       </c>
-      <c r="I106" s="21"/>
-      <c r="J106" s="21"/>
-      <c r="K106" s="21"/>
-      <c r="L106" s="21"/>
-      <c r="M106" s="21"/>
+      <c r="I106" s="15"/>
+      <c r="J106" s="15"/>
+      <c r="K106" s="15"/>
+      <c r="L106" s="15"/>
+      <c r="M106" s="15"/>
     </row>
     <row r="107" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A107" s="3" t="s">
@@ -4332,11 +4329,11 @@
       <c r="H107" s="3">
         <v>13.8</v>
       </c>
-      <c r="I107" s="21"/>
-      <c r="J107" s="21"/>
-      <c r="K107" s="21"/>
-      <c r="L107" s="21"/>
-      <c r="M107" s="21"/>
+      <c r="I107" s="15"/>
+      <c r="J107" s="15"/>
+      <c r="K107" s="15"/>
+      <c r="L107" s="15"/>
+      <c r="M107" s="15"/>
     </row>
     <row r="108" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A108" s="3" t="s">
@@ -4361,15 +4358,15 @@
       <c r="H108" s="3">
         <v>27.16</v>
       </c>
-      <c r="I108" s="21"/>
-      <c r="J108" s="21"/>
-      <c r="K108" s="21">
+      <c r="I108" s="15"/>
+      <c r="J108" s="15"/>
+      <c r="K108" s="15">
         <v>28.3</v>
       </c>
-      <c r="L108" s="21">
+      <c r="L108" s="15">
         <v>19.899999999999999</v>
       </c>
-      <c r="M108" s="21">
+      <c r="M108" s="15">
         <v>3.7</v>
       </c>
     </row>
@@ -4396,11 +4393,11 @@
       <c r="H109" s="3">
         <v>117.74</v>
       </c>
-      <c r="I109" s="21"/>
-      <c r="J109" s="21"/>
-      <c r="K109" s="21"/>
-      <c r="L109" s="21"/>
-      <c r="M109" s="21"/>
+      <c r="I109" s="15"/>
+      <c r="J109" s="15"/>
+      <c r="K109" s="15"/>
+      <c r="L109" s="15"/>
+      <c r="M109" s="15"/>
     </row>
     <row r="110" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A110" s="3" t="s">
@@ -4425,19 +4422,19 @@
       <c r="H110" s="3">
         <v>29.66</v>
       </c>
-      <c r="I110" s="21" t="s">
+      <c r="I110" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J110" s="21">
+      <c r="J110" s="15">
         <v>25.7</v>
       </c>
-      <c r="K110" s="21">
+      <c r="K110" s="15">
         <v>29.1</v>
       </c>
-      <c r="L110" s="21">
+      <c r="L110" s="15">
         <v>23.6</v>
       </c>
-      <c r="M110" s="21">
+      <c r="M110" s="15">
         <v>7.4</v>
       </c>
     </row>
@@ -4466,19 +4463,19 @@
       <c r="H111" s="3">
         <v>32.08</v>
       </c>
-      <c r="I111" s="21" t="s">
+      <c r="I111" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J111" s="21">
+      <c r="J111" s="15">
         <v>31.5</v>
       </c>
-      <c r="K111" s="21">
+      <c r="K111" s="15">
         <v>28.7</v>
       </c>
-      <c r="L111" s="21">
+      <c r="L111" s="15">
         <v>26.4</v>
       </c>
-      <c r="M111" s="21">
+      <c r="M111" s="15">
         <v>8.3000000000000007</v>
       </c>
     </row>
@@ -4505,11 +4502,11 @@
       <c r="H112" s="3">
         <v>17.22</v>
       </c>
-      <c r="I112" s="21"/>
-      <c r="J112" s="21"/>
-      <c r="K112" s="21"/>
-      <c r="L112" s="21"/>
-      <c r="M112" s="21"/>
+      <c r="I112" s="15"/>
+      <c r="J112" s="15"/>
+      <c r="K112" s="15"/>
+      <c r="L112" s="15"/>
+      <c r="M112" s="15"/>
     </row>
     <row r="113" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A113" s="3" t="s">
@@ -4534,11 +4531,11 @@
       <c r="H113" s="3">
         <v>131.69</v>
       </c>
-      <c r="I113" s="21"/>
-      <c r="J113" s="21"/>
-      <c r="K113" s="21"/>
-      <c r="L113" s="21"/>
-      <c r="M113" s="21"/>
+      <c r="I113" s="15"/>
+      <c r="J113" s="15"/>
+      <c r="K113" s="15"/>
+      <c r="L113" s="15"/>
+      <c r="M113" s="15"/>
     </row>
     <row r="114" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A114" s="3" t="s">
@@ -4563,19 +4560,19 @@
       <c r="H114" s="3">
         <v>7.73</v>
       </c>
-      <c r="I114" s="21" t="s">
+      <c r="I114" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J114" s="21">
+      <c r="J114" s="15">
         <v>21.8</v>
       </c>
-      <c r="K114" s="21">
+      <c r="K114" s="15">
         <v>22.8</v>
       </c>
-      <c r="L114" s="21">
+      <c r="L114" s="15">
         <v>26.4</v>
       </c>
-      <c r="M114" s="21">
+      <c r="M114" s="15">
         <v>2.7</v>
       </c>
     </row>
@@ -4602,11 +4599,11 @@
       <c r="H115" s="3">
         <v>18.61</v>
       </c>
-      <c r="I115" s="21"/>
-      <c r="J115" s="21"/>
-      <c r="K115" s="21"/>
-      <c r="L115" s="21"/>
-      <c r="M115" s="21"/>
+      <c r="I115" s="15"/>
+      <c r="J115" s="15"/>
+      <c r="K115" s="15"/>
+      <c r="L115" s="15"/>
+      <c r="M115" s="15"/>
     </row>
     <row r="116" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A116" s="3" t="s">
@@ -4631,11 +4628,11 @@
       <c r="H116" s="3">
         <v>11.75</v>
       </c>
-      <c r="I116" s="21"/>
-      <c r="J116" s="21"/>
-      <c r="K116" s="21"/>
-      <c r="L116" s="21"/>
-      <c r="M116" s="21"/>
+      <c r="I116" s="15"/>
+      <c r="J116" s="15"/>
+      <c r="K116" s="15"/>
+      <c r="L116" s="15"/>
+      <c r="M116" s="15"/>
     </row>
     <row r="117" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A117" s="3" t="s">
@@ -4660,19 +4657,19 @@
       <c r="H117" s="3">
         <v>423.33</v>
       </c>
-      <c r="I117" s="21" t="s">
+      <c r="I117" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J117" s="21">
+      <c r="J117" s="15">
         <v>18.3</v>
       </c>
-      <c r="K117" s="21">
+      <c r="K117" s="15">
         <v>21.6</v>
       </c>
-      <c r="L117" s="21">
+      <c r="L117" s="15">
         <v>11.7</v>
       </c>
-      <c r="M117" s="21">
+      <c r="M117" s="15">
         <v>1.5</v>
       </c>
     </row>
@@ -4697,19 +4694,19 @@
       <c r="H118" s="3">
         <v>394.45</v>
       </c>
-      <c r="I118" s="21" t="s">
+      <c r="I118" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J118" s="21">
+      <c r="J118" s="15">
         <v>19.399999999999999</v>
       </c>
-      <c r="K118" s="21">
+      <c r="K118" s="15">
         <v>23.9</v>
       </c>
-      <c r="L118" s="21">
+      <c r="L118" s="15">
         <v>13.5</v>
       </c>
-      <c r="M118" s="21">
+      <c r="M118" s="15">
         <v>1.2</v>
       </c>
     </row>
@@ -4722,11 +4719,11 @@
       <c r="F119" s="3"/>
       <c r="G119" s="3"/>
       <c r="H119" s="3"/>
-      <c r="I119" s="21"/>
-      <c r="J119" s="21"/>
-      <c r="K119" s="21"/>
-      <c r="L119" s="21"/>
-      <c r="M119" s="21"/>
+      <c r="I119" s="15"/>
+      <c r="J119" s="15"/>
+      <c r="K119" s="15"/>
+      <c r="L119" s="15"/>
+      <c r="M119" s="15"/>
     </row>
     <row r="120" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A120" s="3" t="s">
@@ -4753,19 +4750,19 @@
       <c r="H120" s="3">
         <v>35.49</v>
       </c>
-      <c r="I120" s="21" t="s">
+      <c r="I120" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J120" s="21">
+      <c r="J120" s="15">
         <v>15.4</v>
       </c>
-      <c r="K120" s="21">
+      <c r="K120" s="15">
         <v>20.399999999999999</v>
       </c>
-      <c r="L120" s="21">
+      <c r="L120" s="15">
         <v>4.3</v>
       </c>
-      <c r="M120" s="21">
+      <c r="M120" s="15">
         <v>2.2999999999999998</v>
       </c>
     </row>
@@ -4794,19 +4791,19 @@
       <c r="H121" s="3">
         <v>48.11</v>
       </c>
-      <c r="I121" s="21" t="s">
+      <c r="I121" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J121" s="21">
+      <c r="J121" s="15">
         <v>19.399999999999999</v>
       </c>
-      <c r="K121" s="21">
+      <c r="K121" s="15">
         <v>22.7</v>
       </c>
-      <c r="L121" s="21">
+      <c r="L121" s="15">
         <v>6.4</v>
       </c>
-      <c r="M121" s="21">
+      <c r="M121" s="15">
         <v>1.8</v>
       </c>
     </row>
@@ -4835,19 +4832,19 @@
       <c r="H122" s="3">
         <v>33.299999999999997</v>
       </c>
-      <c r="I122" s="21" t="s">
+      <c r="I122" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J122" s="21">
+      <c r="J122" s="15">
         <v>23.8</v>
       </c>
-      <c r="K122" s="21">
+      <c r="K122" s="15">
         <v>29.6</v>
       </c>
-      <c r="L122" s="21">
+      <c r="L122" s="15">
         <v>24.5</v>
       </c>
-      <c r="M122" s="21">
+      <c r="M122" s="15">
         <v>11.3</v>
       </c>
     </row>
@@ -4876,19 +4873,19 @@
       <c r="H123" s="3">
         <v>48.92</v>
       </c>
-      <c r="I123" s="21" t="s">
+      <c r="I123" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J123" s="21">
+      <c r="J123" s="15">
         <v>17.899999999999999</v>
       </c>
-      <c r="K123" s="21">
+      <c r="K123" s="15">
         <v>20.399999999999999</v>
       </c>
-      <c r="L123" s="21">
+      <c r="L123" s="15">
         <v>9.3000000000000007</v>
       </c>
-      <c r="M123" s="21">
+      <c r="M123" s="15">
         <v>1.4</v>
       </c>
     </row>
@@ -4915,19 +4912,19 @@
       <c r="H124" s="3">
         <v>39.659999999999997</v>
       </c>
-      <c r="I124" s="21" t="s">
+      <c r="I124" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J124" s="21">
+      <c r="J124" s="15">
         <v>18.566600000000001</v>
       </c>
-      <c r="K124" s="21">
+      <c r="K124" s="15">
         <v>20.8</v>
       </c>
-      <c r="L124" s="21">
+      <c r="L124" s="15">
         <v>3.09</v>
       </c>
-      <c r="M124" s="21">
+      <c r="M124" s="15">
         <v>0.9</v>
       </c>
     </row>
@@ -4954,19 +4951,19 @@
       <c r="H125" s="3">
         <v>40.06</v>
       </c>
-      <c r="I125" s="21" t="s">
+      <c r="I125" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J125" s="21">
+      <c r="J125" s="15">
         <v>19.3</v>
       </c>
-      <c r="K125" s="21">
+      <c r="K125" s="15">
         <v>17.5</v>
       </c>
-      <c r="L125" s="21">
+      <c r="L125" s="15">
         <v>7.4</v>
       </c>
-      <c r="M125" s="21">
+      <c r="M125" s="15">
         <v>0.7</v>
       </c>
     </row>
@@ -4993,11 +4990,11 @@
       <c r="H126" s="3">
         <v>17.440000000000001</v>
       </c>
-      <c r="I126" s="21"/>
-      <c r="J126" s="21"/>
-      <c r="K126" s="21"/>
-      <c r="L126" s="21"/>
-      <c r="M126" s="21"/>
+      <c r="I126" s="15"/>
+      <c r="J126" s="15"/>
+      <c r="K126" s="15"/>
+      <c r="L126" s="15"/>
+      <c r="M126" s="15"/>
     </row>
     <row r="127" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A127" s="3" t="s">
@@ -5022,19 +5019,19 @@
       <c r="H127" s="3">
         <v>221.16</v>
       </c>
-      <c r="I127" s="21" t="s">
+      <c r="I127" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J127" s="21">
+      <c r="J127" s="15">
         <v>7.6</v>
       </c>
-      <c r="K127" s="21">
+      <c r="K127" s="15">
         <v>22.4</v>
       </c>
-      <c r="L127" s="21">
+      <c r="L127" s="15">
         <v>9.3000000000000007</v>
       </c>
-      <c r="M127" s="21">
+      <c r="M127" s="15">
         <v>2.1</v>
       </c>
     </row>
@@ -5061,11 +5058,11 @@
       <c r="H128" s="3">
         <v>16.989999999999998</v>
       </c>
-      <c r="I128" s="21"/>
-      <c r="J128" s="21"/>
-      <c r="K128" s="21"/>
-      <c r="L128" s="21"/>
-      <c r="M128" s="21"/>
+      <c r="I128" s="15"/>
+      <c r="J128" s="15"/>
+      <c r="K128" s="15"/>
+      <c r="L128" s="15"/>
+      <c r="M128" s="15"/>
     </row>
     <row r="129" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A129" s="3" t="s">
@@ -5090,11 +5087,11 @@
       <c r="H129" s="3">
         <v>8.32</v>
       </c>
-      <c r="I129" s="21"/>
-      <c r="J129" s="21"/>
-      <c r="K129" s="21"/>
-      <c r="L129" s="21"/>
-      <c r="M129" s="21"/>
+      <c r="I129" s="15"/>
+      <c r="J129" s="15"/>
+      <c r="K129" s="15"/>
+      <c r="L129" s="15"/>
+      <c r="M129" s="15"/>
     </row>
     <row r="130" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A130" s="3" t="s">
@@ -5121,13 +5118,13 @@
       <c r="H130" s="3">
         <v>37.15</v>
       </c>
-      <c r="I130" s="21"/>
-      <c r="J130" s="21"/>
-      <c r="K130" s="21"/>
-      <c r="L130" s="21">
+      <c r="I130" s="15"/>
+      <c r="J130" s="15"/>
+      <c r="K130" s="15"/>
+      <c r="L130" s="15">
         <v>2.0299999999999998</v>
       </c>
-      <c r="M130" s="21"/>
+      <c r="M130" s="15"/>
     </row>
     <row r="131" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A131" s="3" t="s">
@@ -5154,11 +5151,11 @@
       <c r="H131" s="3">
         <v>32.06</v>
       </c>
-      <c r="I131" s="21"/>
-      <c r="J131" s="21"/>
-      <c r="K131" s="21"/>
-      <c r="L131" s="21"/>
-      <c r="M131" s="21"/>
+      <c r="I131" s="15"/>
+      <c r="J131" s="15"/>
+      <c r="K131" s="15"/>
+      <c r="L131" s="15"/>
+      <c r="M131" s="15"/>
     </row>
     <row r="132" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A132" s="3" t="s">
@@ -5185,19 +5182,19 @@
       <c r="H132" s="3">
         <v>31.08</v>
       </c>
-      <c r="I132" s="21" t="s">
+      <c r="I132" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J132" s="21">
+      <c r="J132" s="15">
         <v>5.4</v>
       </c>
-      <c r="K132" s="21">
+      <c r="K132" s="15">
         <v>19.7</v>
       </c>
-      <c r="L132" s="21">
+      <c r="L132" s="15">
         <v>3.3</v>
       </c>
-      <c r="M132" s="21">
+      <c r="M132" s="15">
         <v>0.66</v>
       </c>
     </row>
@@ -5224,19 +5221,19 @@
       <c r="H133" s="3">
         <v>47.71</v>
       </c>
-      <c r="I133" s="21" t="s">
+      <c r="I133" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J133" s="21">
+      <c r="J133" s="15">
         <v>9.4</v>
       </c>
-      <c r="K133" s="21">
+      <c r="K133" s="15">
         <v>21.5</v>
       </c>
-      <c r="L133" s="21">
+      <c r="L133" s="15">
         <v>4.5</v>
       </c>
-      <c r="M133" s="21">
+      <c r="M133" s="15">
         <v>0.9</v>
       </c>
     </row>
@@ -5263,11 +5260,11 @@
       <c r="H134" s="3">
         <v>36.54</v>
       </c>
-      <c r="I134" s="21"/>
-      <c r="J134" s="21"/>
-      <c r="K134" s="21"/>
-      <c r="L134" s="21"/>
-      <c r="M134" s="21"/>
+      <c r="I134" s="15"/>
+      <c r="J134" s="15"/>
+      <c r="K134" s="15"/>
+      <c r="L134" s="15"/>
+      <c r="M134" s="15"/>
     </row>
     <row r="135" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A135" s="3" t="s">
@@ -5292,11 +5289,11 @@
       <c r="H135" s="3">
         <v>30.9</v>
       </c>
-      <c r="I135" s="21"/>
-      <c r="J135" s="21"/>
-      <c r="K135" s="21"/>
-      <c r="L135" s="21"/>
-      <c r="M135" s="21"/>
+      <c r="I135" s="15"/>
+      <c r="J135" s="15"/>
+      <c r="K135" s="15"/>
+      <c r="L135" s="15"/>
+      <c r="M135" s="15"/>
     </row>
     <row r="136" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A136" s="3" t="s">
@@ -5321,11 +5318,11 @@
       <c r="H136" s="3">
         <v>7.8</v>
       </c>
-      <c r="I136" s="21"/>
-      <c r="J136" s="21"/>
-      <c r="K136" s="21"/>
-      <c r="L136" s="21"/>
-      <c r="M136" s="21"/>
+      <c r="I136" s="15"/>
+      <c r="J136" s="15"/>
+      <c r="K136" s="15"/>
+      <c r="L136" s="15"/>
+      <c r="M136" s="15"/>
     </row>
     <row r="137" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A137" s="3" t="s">
@@ -5352,19 +5349,19 @@
       <c r="H137" s="3">
         <v>36.700000000000003</v>
       </c>
-      <c r="I137" s="21" t="s">
+      <c r="I137" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J137" s="21">
+      <c r="J137" s="15">
         <v>11.4</v>
       </c>
-      <c r="K137" s="21">
+      <c r="K137" s="15">
         <v>23.4</v>
       </c>
-      <c r="L137" s="21">
+      <c r="L137" s="15">
         <v>4.4000000000000004</v>
       </c>
-      <c r="M137" s="21">
+      <c r="M137" s="15">
         <v>0.55000000000000004</v>
       </c>
     </row>
@@ -5393,19 +5390,19 @@
       <c r="H138" s="3">
         <v>31.54</v>
       </c>
-      <c r="I138" s="21" t="s">
+      <c r="I138" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J138" s="21">
+      <c r="J138" s="15">
         <v>10.3</v>
       </c>
-      <c r="K138" s="21">
+      <c r="K138" s="15">
         <v>26.4</v>
       </c>
-      <c r="L138" s="21">
+      <c r="L138" s="15">
         <v>7.3</v>
       </c>
-      <c r="M138" s="21">
+      <c r="M138" s="15">
         <v>1.03</v>
       </c>
     </row>
@@ -5434,19 +5431,19 @@
       <c r="H139" s="3">
         <v>22.59</v>
       </c>
-      <c r="I139" s="21" t="s">
+      <c r="I139" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J139" s="21">
+      <c r="J139" s="15">
         <v>3.9</v>
       </c>
-      <c r="K139" s="21">
+      <c r="K139" s="15">
         <v>19.899999999999999</v>
       </c>
-      <c r="L139" s="21">
+      <c r="L139" s="15">
         <v>8.3000000000000007</v>
       </c>
-      <c r="M139" s="21">
+      <c r="M139" s="15">
         <v>0.65</v>
       </c>
     </row>
@@ -5475,11 +5472,11 @@
       <c r="H140" s="3">
         <v>45.33</v>
       </c>
-      <c r="I140" s="21"/>
-      <c r="J140" s="21"/>
-      <c r="K140" s="21"/>
-      <c r="L140" s="21"/>
-      <c r="M140" s="21"/>
+      <c r="I140" s="15"/>
+      <c r="J140" s="15"/>
+      <c r="K140" s="15"/>
+      <c r="L140" s="15"/>
+      <c r="M140" s="15"/>
     </row>
     <row r="141" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A141" s="3" t="s">
@@ -5506,11 +5503,11 @@
       <c r="H141" s="3">
         <v>35.049999999999997</v>
       </c>
-      <c r="I141" s="21"/>
-      <c r="J141" s="21"/>
-      <c r="K141" s="21"/>
-      <c r="L141" s="21"/>
-      <c r="M141" s="21"/>
+      <c r="I141" s="15"/>
+      <c r="J141" s="15"/>
+      <c r="K141" s="15"/>
+      <c r="L141" s="15"/>
+      <c r="M141" s="15"/>
     </row>
     <row r="142" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A142" s="3" t="s">
@@ -5537,12 +5534,12 @@
       <c r="H142" s="3">
         <v>33.99</v>
       </c>
-      <c r="I142" s="21"/>
-      <c r="J142" s="21"/>
-      <c r="L142" s="21">
+      <c r="I142" s="15"/>
+      <c r="J142" s="15"/>
+      <c r="L142" s="15">
         <v>3.3</v>
       </c>
-      <c r="M142" s="21"/>
+      <c r="M142" s="15"/>
     </row>
     <row r="143" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A143" s="3" t="s">
@@ -5567,19 +5564,19 @@
       <c r="H143" s="3">
         <v>6.08</v>
       </c>
-      <c r="I143" s="21" t="s">
+      <c r="I143" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J143" s="21">
+      <c r="J143" s="15">
         <v>15.9</v>
       </c>
-      <c r="K143" s="21">
+      <c r="K143" s="15">
         <v>28.4</v>
       </c>
-      <c r="L143" s="21">
+      <c r="L143" s="15">
         <v>12.3</v>
       </c>
-      <c r="M143" s="21">
+      <c r="M143" s="15">
         <v>11.4</v>
       </c>
     </row>
@@ -5606,19 +5603,19 @@
       <c r="H144" s="3">
         <v>196.75</v>
       </c>
-      <c r="I144" s="21" t="s">
+      <c r="I144" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J144" s="21">
+      <c r="J144" s="15">
         <v>3.9</v>
       </c>
-      <c r="K144" s="21">
+      <c r="K144" s="15">
         <v>21.8</v>
       </c>
-      <c r="L144" s="21">
+      <c r="L144" s="15">
         <v>9.1999999999999993</v>
       </c>
-      <c r="M144" s="21">
+      <c r="M144" s="15">
         <v>2.7</v>
       </c>
     </row>
@@ -5647,19 +5644,19 @@
       <c r="H145" s="3">
         <v>46.44</v>
       </c>
-      <c r="I145" s="21" t="s">
+      <c r="I145" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J145" s="21">
+      <c r="J145" s="15">
         <v>15.3</v>
       </c>
-      <c r="K145" s="21">
+      <c r="K145" s="15">
         <v>25.8</v>
       </c>
-      <c r="L145" s="21">
+      <c r="L145" s="15">
         <v>21.3</v>
       </c>
-      <c r="M145" s="21">
+      <c r="M145" s="15">
         <v>10.8</v>
       </c>
     </row>
@@ -5686,19 +5683,19 @@
       <c r="H146" s="3">
         <v>175.9</v>
       </c>
-      <c r="I146" s="21" t="s">
+      <c r="I146" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J146" s="21">
+      <c r="J146" s="15">
         <v>5.9</v>
       </c>
-      <c r="K146" s="21">
+      <c r="K146" s="15">
         <v>20.399999999999999</v>
       </c>
-      <c r="L146" s="21">
+      <c r="L146" s="15">
         <v>11.2</v>
       </c>
-      <c r="M146" s="21">
+      <c r="M146" s="15">
         <v>2.7</v>
       </c>
     </row>
@@ -5725,11 +5722,11 @@
       <c r="H147" s="3">
         <v>213.7</v>
       </c>
-      <c r="I147" s="21"/>
-      <c r="J147" s="21"/>
-      <c r="K147" s="21"/>
-      <c r="L147" s="21"/>
-      <c r="M147" s="21"/>
+      <c r="I147" s="15"/>
+      <c r="J147" s="15"/>
+      <c r="K147" s="15"/>
+      <c r="L147" s="15"/>
+      <c r="M147" s="15"/>
     </row>
     <row r="148" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A148" s="3" t="s">
@@ -5754,19 +5751,19 @@
       <c r="H148" s="3">
         <v>273.5</v>
       </c>
-      <c r="I148" s="21" t="s">
+      <c r="I148" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J148" s="21">
+      <c r="J148" s="15">
         <v>8.5</v>
       </c>
-      <c r="K148" s="21">
+      <c r="K148" s="15">
         <v>23.8</v>
       </c>
-      <c r="L148" s="21">
+      <c r="L148" s="15">
         <v>3.6</v>
       </c>
-      <c r="M148" s="21">
+      <c r="M148" s="15">
         <v>2.1</v>
       </c>
     </row>
@@ -5791,19 +5788,19 @@
       <c r="H149" s="3">
         <v>810.5</v>
       </c>
-      <c r="I149" s="21" t="s">
+      <c r="I149" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J149" s="21">
+      <c r="J149" s="15">
         <v>11.7</v>
       </c>
-      <c r="K149" s="21">
+      <c r="K149" s="15">
         <v>22.6</v>
       </c>
-      <c r="L149" s="21">
+      <c r="L149" s="15">
         <v>7.3</v>
       </c>
-      <c r="M149" s="21">
+      <c r="M149" s="15">
         <v>3.4</v>
       </c>
     </row>
@@ -5830,19 +5827,19 @@
       <c r="H150" s="3">
         <v>9.6</v>
       </c>
-      <c r="I150" s="21" t="s">
+      <c r="I150" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J150" s="21">
+      <c r="J150" s="15">
         <v>32.6</v>
       </c>
-      <c r="K150" s="21">
+      <c r="K150" s="15">
         <v>29.6</v>
       </c>
-      <c r="L150" s="21">
+      <c r="L150" s="15">
         <v>22.7</v>
       </c>
-      <c r="M150" s="21">
+      <c r="M150" s="15">
         <v>12.8</v>
       </c>
     </row>
@@ -5869,15 +5866,15 @@
       <c r="H151" s="3">
         <v>34.700000000000003</v>
       </c>
-      <c r="I151" s="21" t="s">
+      <c r="I151" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J151" s="21"/>
-      <c r="K151" s="21"/>
-      <c r="L151" s="21">
+      <c r="J151" s="15"/>
+      <c r="K151" s="15"/>
+      <c r="L151" s="15">
         <v>19.3</v>
       </c>
-      <c r="M151" s="21">
+      <c r="M151" s="15">
         <v>0.91</v>
       </c>
     </row>
@@ -5906,19 +5903,19 @@
       <c r="H152" s="3">
         <v>17.579999999999998</v>
       </c>
-      <c r="I152" s="21" t="s">
+      <c r="I152" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J152" s="21">
+      <c r="J152" s="15">
         <v>7.3</v>
       </c>
-      <c r="K152" s="21">
+      <c r="K152" s="15">
         <v>23.4</v>
       </c>
-      <c r="L152" s="21">
+      <c r="L152" s="15">
         <v>12.66</v>
       </c>
-      <c r="M152" s="21">
+      <c r="M152" s="15">
         <v>7.8E-2</v>
       </c>
     </row>
@@ -5947,19 +5944,19 @@
       <c r="H153" s="3">
         <v>4.58</v>
       </c>
-      <c r="I153" s="21" t="s">
+      <c r="I153" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J153" s="21">
+      <c r="J153" s="15">
         <v>6.39</v>
       </c>
-      <c r="K153" s="21">
+      <c r="K153" s="15">
         <v>20.399999999999999</v>
       </c>
-      <c r="L153" s="21">
+      <c r="L153" s="15">
         <v>3.8</v>
       </c>
-      <c r="M153" s="21">
+      <c r="M153" s="15">
         <v>0.3</v>
       </c>
     </row>
@@ -5988,19 +5985,19 @@
       <c r="H154" s="3">
         <v>30.16</v>
       </c>
-      <c r="I154" s="21" t="s">
+      <c r="I154" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J154" s="21">
+      <c r="J154" s="15">
         <v>6.9</v>
       </c>
-      <c r="K154" s="21">
+      <c r="K154" s="15">
         <v>19.5</v>
       </c>
-      <c r="L154" s="21">
+      <c r="L154" s="15">
         <v>4.3</v>
       </c>
-      <c r="M154" s="21">
+      <c r="M154" s="15">
         <v>0.24</v>
       </c>
     </row>
@@ -6029,19 +6026,19 @@
       <c r="H155" s="3">
         <v>31.35</v>
       </c>
-      <c r="I155" s="21" t="s">
+      <c r="I155" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J155" s="21">
+      <c r="J155" s="15">
         <v>5.6</v>
       </c>
-      <c r="K155" s="21">
+      <c r="K155" s="15">
         <v>20.5</v>
       </c>
-      <c r="L155" s="21">
+      <c r="L155" s="15">
         <v>7.1</v>
       </c>
-      <c r="M155" s="21">
+      <c r="M155" s="15">
         <v>0.6</v>
       </c>
     </row>
@@ -6070,19 +6067,19 @@
       <c r="H156" s="3">
         <v>32.29</v>
       </c>
-      <c r="I156" s="21" t="s">
+      <c r="I156" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J156" s="21">
+      <c r="J156" s="15">
         <v>3.9</v>
       </c>
-      <c r="K156" s="21">
+      <c r="K156" s="15">
         <v>23.1</v>
       </c>
-      <c r="L156" s="21">
+      <c r="L156" s="15">
         <v>4.9000000000000004</v>
       </c>
-      <c r="M156" s="21">
+      <c r="M156" s="15">
         <v>0.3</v>
       </c>
     </row>
@@ -6111,19 +6108,19 @@
       <c r="H157" s="3">
         <v>29.2</v>
       </c>
-      <c r="I157" s="21" t="s">
+      <c r="I157" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J157" s="21">
+      <c r="J157" s="15">
         <v>9.3000000000000007</v>
       </c>
-      <c r="K157" s="21">
+      <c r="K157" s="15">
         <v>24.2</v>
       </c>
-      <c r="L157" s="21">
+      <c r="L157" s="15">
         <v>3.8</v>
       </c>
-      <c r="M157" s="21">
+      <c r="M157" s="15">
         <v>0.23</v>
       </c>
     </row>
@@ -6152,19 +6149,19 @@
       <c r="H158" s="3">
         <v>15.2</v>
       </c>
-      <c r="I158" s="21" t="s">
+      <c r="I158" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J158" s="21">
+      <c r="J158" s="15">
         <v>2.7</v>
       </c>
-      <c r="K158" s="21">
+      <c r="K158" s="15">
         <v>20.2</v>
       </c>
-      <c r="L158" s="21">
+      <c r="L158" s="15">
         <v>5.4</v>
       </c>
-      <c r="M158" s="21">
+      <c r="M158" s="15">
         <v>0.76</v>
       </c>
     </row>
@@ -6193,19 +6190,19 @@
       <c r="H159" s="3">
         <v>38.85</v>
       </c>
-      <c r="I159" s="21" t="s">
+      <c r="I159" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J159" s="21">
+      <c r="J159" s="15">
         <v>6.2</v>
       </c>
-      <c r="K159" s="21">
+      <c r="K159" s="15">
         <v>22.4</v>
       </c>
-      <c r="L159" s="21">
+      <c r="L159" s="15">
         <v>4.4000000000000004</v>
       </c>
-      <c r="M159" s="21">
+      <c r="M159" s="15">
         <v>0.33</v>
       </c>
     </row>
@@ -6234,11 +6231,11 @@
       <c r="H160" s="3">
         <v>20.7</v>
       </c>
-      <c r="I160" s="21"/>
-      <c r="J160" s="21"/>
-      <c r="K160" s="21"/>
-      <c r="L160" s="21"/>
-      <c r="M160" s="21"/>
+      <c r="I160" s="15"/>
+      <c r="J160" s="15"/>
+      <c r="K160" s="15"/>
+      <c r="L160" s="15"/>
+      <c r="M160" s="15"/>
     </row>
     <row r="161" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A161" s="3" t="s">
@@ -6265,11 +6262,11 @@
       <c r="H161" s="3">
         <v>39.83</v>
       </c>
-      <c r="I161" s="21"/>
-      <c r="J161" s="21"/>
-      <c r="K161" s="21"/>
-      <c r="L161" s="21"/>
-      <c r="M161" s="21"/>
+      <c r="I161" s="15"/>
+      <c r="J161" s="15"/>
+      <c r="K161" s="15"/>
+      <c r="L161" s="15"/>
+      <c r="M161" s="15"/>
     </row>
     <row r="162" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A162" s="3" t="s">
@@ -6296,19 +6293,19 @@
       <c r="H162" s="3">
         <v>42.42</v>
       </c>
-      <c r="I162" s="21" t="s">
+      <c r="I162" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J162" s="21">
+      <c r="J162" s="15">
         <v>14.3</v>
       </c>
-      <c r="K162" s="21">
+      <c r="K162" s="15">
         <v>27.5</v>
       </c>
-      <c r="L162" s="21">
+      <c r="L162" s="15">
         <v>14.6</v>
       </c>
-      <c r="M162" s="21">
+      <c r="M162" s="15">
         <v>11.23</v>
       </c>
     </row>
@@ -6337,19 +6334,19 @@
       <c r="H163" s="3">
         <v>28.73</v>
       </c>
-      <c r="I163" s="21" t="s">
+      <c r="I163" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J163" s="21">
+      <c r="J163" s="15">
         <v>13.2</v>
       </c>
-      <c r="K163" s="21">
+      <c r="K163" s="15">
         <v>31.4</v>
       </c>
-      <c r="L163" s="21">
+      <c r="L163" s="15">
         <v>15.2</v>
       </c>
-      <c r="M163" s="21">
+      <c r="M163" s="15">
         <v>12.7</v>
       </c>
     </row>
@@ -6378,19 +6375,19 @@
       <c r="H164" s="3">
         <v>26.32</v>
       </c>
-      <c r="I164" s="21" t="s">
+      <c r="I164" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J164" s="21">
+      <c r="J164" s="15">
         <v>9.3000000000000007</v>
       </c>
-      <c r="K164" s="21">
+      <c r="K164" s="15">
         <v>26.8</v>
       </c>
-      <c r="L164" s="21">
+      <c r="L164" s="15">
         <v>7.2</v>
       </c>
-      <c r="M164" s="21">
+      <c r="M164" s="15">
         <v>12.3</v>
       </c>
     </row>
@@ -6419,19 +6416,19 @@
       <c r="H165" s="3">
         <v>17.920000000000002</v>
       </c>
-      <c r="I165" s="21" t="s">
+      <c r="I165" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J165" s="21">
+      <c r="J165" s="15">
         <v>8.1999999999999993</v>
       </c>
-      <c r="K165" s="21">
+      <c r="K165" s="15">
         <v>25.3</v>
       </c>
-      <c r="L165" s="21">
+      <c r="L165" s="15">
         <v>5.8</v>
       </c>
-      <c r="M165" s="21">
+      <c r="M165" s="15">
         <v>12.4</v>
       </c>
     </row>
@@ -6458,11 +6455,11 @@
       <c r="H166" s="3">
         <v>21.84</v>
       </c>
-      <c r="I166" s="21"/>
-      <c r="J166" s="21"/>
-      <c r="K166" s="21"/>
-      <c r="L166" s="21"/>
-      <c r="M166" s="21"/>
+      <c r="I166" s="15"/>
+      <c r="J166" s="15"/>
+      <c r="K166" s="15"/>
+      <c r="L166" s="15"/>
+      <c r="M166" s="15"/>
     </row>
     <row r="167" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A167" s="3" t="s">
@@ -6487,11 +6484,11 @@
       <c r="H167" s="3">
         <v>11.72</v>
       </c>
-      <c r="I167" s="21"/>
-      <c r="J167" s="21"/>
-      <c r="K167" s="21"/>
-      <c r="L167" s="21"/>
-      <c r="M167" s="21"/>
+      <c r="I167" s="15"/>
+      <c r="J167" s="15"/>
+      <c r="K167" s="15"/>
+      <c r="L167" s="15"/>
+      <c r="M167" s="15"/>
     </row>
     <row r="168" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A168" s="3" t="s">
@@ -6516,19 +6513,19 @@
       <c r="H168" s="3">
         <v>9.4499999999999993</v>
       </c>
-      <c r="I168" s="21" t="s">
+      <c r="I168" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J168" s="21">
+      <c r="J168" s="15">
         <v>11.5</v>
       </c>
-      <c r="K168" s="21">
+      <c r="K168" s="15">
         <v>29.7</v>
       </c>
-      <c r="L168" s="21">
+      <c r="L168" s="15">
         <v>14.2</v>
       </c>
-      <c r="M168" s="21">
+      <c r="M168" s="15">
         <v>13.3</v>
       </c>
     </row>
@@ -6557,11 +6554,11 @@
       <c r="H169" s="3">
         <v>29.89</v>
       </c>
-      <c r="I169" s="21"/>
-      <c r="J169" s="21"/>
-      <c r="K169" s="21"/>
-      <c r="L169" s="21"/>
-      <c r="M169" s="21"/>
+      <c r="I169" s="15"/>
+      <c r="J169" s="15"/>
+      <c r="K169" s="15"/>
+      <c r="L169" s="15"/>
+      <c r="M169" s="15"/>
     </row>
     <row r="170" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A170" s="3" t="s">
@@ -6588,19 +6585,19 @@
       <c r="H170" s="3">
         <v>33.07</v>
       </c>
-      <c r="I170" s="21" t="s">
+      <c r="I170" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J170" s="21">
+      <c r="J170" s="15">
         <v>12.7</v>
       </c>
-      <c r="K170" s="21">
+      <c r="K170" s="15">
         <v>31.4</v>
       </c>
-      <c r="L170" s="21">
+      <c r="L170" s="15">
         <v>18.2</v>
       </c>
-      <c r="M170" s="21">
+      <c r="M170" s="15">
         <v>14.2</v>
       </c>
     </row>
@@ -6629,19 +6626,19 @@
       <c r="H171" s="3">
         <v>33.979999999999997</v>
       </c>
-      <c r="I171" s="21" t="s">
+      <c r="I171" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J171" s="21">
+      <c r="J171" s="15">
         <v>9.1999999999999993</v>
       </c>
-      <c r="K171" s="21">
+      <c r="K171" s="15">
         <v>25.4</v>
       </c>
-      <c r="L171" s="21">
+      <c r="L171" s="15">
         <v>9.3000000000000007</v>
       </c>
-      <c r="M171" s="21">
+      <c r="M171" s="15">
         <v>9.1999999999999993</v>
       </c>
     </row>
@@ -6670,19 +6667,19 @@
       <c r="H172" s="3">
         <v>32.1</v>
       </c>
-      <c r="I172" s="21" t="s">
+      <c r="I172" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J172" s="21">
+      <c r="J172" s="15">
         <v>7.5</v>
       </c>
-      <c r="K172" s="21">
+      <c r="K172" s="15">
         <v>24.7</v>
       </c>
-      <c r="L172" s="21">
+      <c r="L172" s="15">
         <v>8.4</v>
       </c>
-      <c r="M172" s="21">
+      <c r="M172" s="15">
         <v>7.7</v>
       </c>
     </row>
@@ -6709,19 +6706,19 @@
       <c r="H173" s="3">
         <v>959.8</v>
       </c>
-      <c r="I173" s="21" t="s">
+      <c r="I173" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J173" s="21">
+      <c r="J173" s="15">
         <v>6.3</v>
       </c>
-      <c r="K173" s="21">
+      <c r="K173" s="15">
         <v>23.6</v>
       </c>
-      <c r="L173" s="21">
+      <c r="L173" s="15">
         <v>4.9000000000000004</v>
       </c>
-      <c r="M173" s="21">
+      <c r="M173" s="15">
         <v>7.5</v>
       </c>
     </row>
@@ -6750,19 +6747,19 @@
       <c r="H174" s="3">
         <v>29.8</v>
       </c>
-      <c r="I174" s="21" t="s">
+      <c r="I174" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J174" s="21">
+      <c r="J174" s="15">
         <v>6.4</v>
       </c>
-      <c r="K174" s="21">
+      <c r="K174" s="15">
         <v>22.4</v>
       </c>
-      <c r="L174" s="21">
+      <c r="L174" s="15">
         <v>5.7</v>
       </c>
-      <c r="M174" s="21">
+      <c r="M174" s="15">
         <v>6.1</v>
       </c>
     </row>
@@ -6791,19 +6788,19 @@
       <c r="H175" s="3">
         <v>28.7</v>
       </c>
-      <c r="I175" s="21" t="s">
+      <c r="I175" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J175" s="21">
+      <c r="J175" s="15">
         <v>6.8</v>
       </c>
-      <c r="K175" s="21">
+      <c r="K175" s="15">
         <v>23.7</v>
       </c>
-      <c r="L175" s="21">
+      <c r="L175" s="15">
         <v>3.34</v>
       </c>
-      <c r="M175" s="21">
+      <c r="M175" s="15">
         <v>0.5</v>
       </c>
     </row>
@@ -6832,19 +6829,19 @@
       <c r="H176" s="3">
         <v>24.8</v>
       </c>
-      <c r="I176" s="21" t="s">
+      <c r="I176" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J176" s="21">
+      <c r="J176" s="15">
         <v>5.8</v>
       </c>
-      <c r="K176" s="21">
+      <c r="K176" s="15">
         <v>24.6</v>
       </c>
-      <c r="L176" s="21">
+      <c r="L176" s="15">
         <v>8.3000000000000007</v>
       </c>
-      <c r="M176" s="21">
+      <c r="M176" s="15">
         <v>2.2999999999999998</v>
       </c>
     </row>
@@ -6871,19 +6868,19 @@
       <c r="H177" s="3">
         <v>10.6</v>
       </c>
-      <c r="I177" s="21" t="s">
+      <c r="I177" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J177" s="21">
+      <c r="J177" s="15">
         <v>9.9</v>
       </c>
-      <c r="K177" s="21">
+      <c r="K177" s="15">
         <v>29.8</v>
       </c>
-      <c r="L177" s="21">
+      <c r="L177" s="15">
         <v>13.5</v>
       </c>
-      <c r="M177" s="21">
+      <c r="M177" s="15">
         <v>6.4</v>
       </c>
     </row>
@@ -6910,19 +6907,19 @@
       <c r="H178" s="3">
         <v>15.6</v>
       </c>
-      <c r="I178" s="21" t="s">
+      <c r="I178" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J178" s="21">
+      <c r="J178" s="15">
         <v>15.6</v>
       </c>
-      <c r="K178" s="21">
+      <c r="K178" s="15">
         <v>32.799999999999997</v>
       </c>
-      <c r="L178" s="21">
+      <c r="L178" s="15">
         <v>14.3</v>
       </c>
-      <c r="M178" s="21">
+      <c r="M178" s="15">
         <v>7.3</v>
       </c>
     </row>
@@ -6949,11 +6946,11 @@
       <c r="H179" s="3">
         <v>29.5</v>
       </c>
-      <c r="I179" s="21"/>
-      <c r="J179" s="21"/>
-      <c r="K179" s="21"/>
-      <c r="L179" s="21"/>
-      <c r="M179" s="21"/>
+      <c r="I179" s="15"/>
+      <c r="J179" s="15"/>
+      <c r="K179" s="15"/>
+      <c r="L179" s="15"/>
+      <c r="M179" s="15"/>
     </row>
     <row r="180" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A180" s="2">
@@ -6978,11 +6975,11 @@
       <c r="H180" s="3">
         <v>34.1</v>
       </c>
-      <c r="I180" s="21"/>
-      <c r="J180" s="21"/>
-      <c r="K180" s="21"/>
-      <c r="L180" s="21"/>
-      <c r="M180" s="21"/>
+      <c r="I180" s="15"/>
+      <c r="J180" s="15"/>
+      <c r="K180" s="15"/>
+      <c r="L180" s="15"/>
+      <c r="M180" s="15"/>
     </row>
     <row r="181" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A181" s="2">
@@ -7009,19 +7006,19 @@
       <c r="H181" s="3">
         <v>250.9</v>
       </c>
-      <c r="I181" s="21" t="s">
+      <c r="I181" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J181" s="21">
+      <c r="J181" s="15">
         <v>6.3</v>
       </c>
-      <c r="K181" s="21">
+      <c r="K181" s="15">
         <v>19.899999999999999</v>
       </c>
-      <c r="L181" s="21">
+      <c r="L181" s="15">
         <v>7.7</v>
       </c>
-      <c r="M181" s="21">
+      <c r="M181" s="15">
         <v>0.3</v>
       </c>
     </row>
@@ -7050,11 +7047,11 @@
       <c r="H182" s="3">
         <v>26.8</v>
       </c>
-      <c r="I182" s="21"/>
-      <c r="J182" s="21"/>
-      <c r="K182" s="21"/>
-      <c r="L182" s="21"/>
-      <c r="M182" s="21"/>
+      <c r="I182" s="15"/>
+      <c r="J182" s="15"/>
+      <c r="K182" s="15"/>
+      <c r="L182" s="15"/>
+      <c r="M182" s="15"/>
     </row>
     <row r="183" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A183" s="2">
@@ -7081,19 +7078,19 @@
       <c r="H183" s="3">
         <v>17.5</v>
       </c>
-      <c r="I183" s="21" t="s">
+      <c r="I183" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J183" s="21">
+      <c r="J183" s="15">
         <v>12.6</v>
       </c>
-      <c r="K183" s="21">
+      <c r="K183" s="15">
         <v>25.7</v>
       </c>
-      <c r="L183" s="21">
+      <c r="L183" s="15">
         <v>13.5</v>
       </c>
-      <c r="M183" s="21">
+      <c r="M183" s="15">
         <v>5.9</v>
       </c>
     </row>
@@ -7122,19 +7119,19 @@
       <c r="H184" s="3">
         <v>24.8</v>
       </c>
-      <c r="I184" s="21" t="s">
+      <c r="I184" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J184" s="21">
+      <c r="J184" s="15">
         <v>15</v>
       </c>
-      <c r="K184" s="21">
+      <c r="K184" s="15">
         <v>28.3</v>
       </c>
-      <c r="L184" s="21">
+      <c r="L184" s="15">
         <v>21.3</v>
       </c>
-      <c r="M184" s="21">
+      <c r="M184" s="15">
         <v>7.8</v>
       </c>
     </row>
@@ -7161,19 +7158,19 @@
       <c r="H185" s="3">
         <v>26.6</v>
       </c>
-      <c r="I185" s="21" t="s">
+      <c r="I185" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J185" s="21">
+      <c r="J185" s="15">
         <v>19</v>
       </c>
-      <c r="K185" s="21">
+      <c r="K185" s="15">
         <v>29.3</v>
       </c>
-      <c r="L185" s="21">
+      <c r="L185" s="15">
         <v>23.7</v>
       </c>
-      <c r="M185" s="21">
+      <c r="M185" s="15">
         <v>10.4</v>
       </c>
     </row>
@@ -7200,19 +7197,19 @@
       <c r="H186" s="3">
         <v>94.8</v>
       </c>
-      <c r="I186" s="21" t="s">
+      <c r="I186" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J186" s="21">
+      <c r="J186" s="15">
         <v>26.6</v>
       </c>
-      <c r="K186" s="21">
+      <c r="K186" s="15">
         <v>31.9</v>
       </c>
-      <c r="L186" s="21">
+      <c r="L186" s="15">
         <v>29.7</v>
       </c>
-      <c r="M186" s="21">
+      <c r="M186" s="15">
         <v>12.6</v>
       </c>
     </row>
@@ -7239,13 +7236,13 @@
       <c r="H187" s="3">
         <v>99.1</v>
       </c>
-      <c r="I187" s="21"/>
-      <c r="J187" s="21"/>
-      <c r="K187" s="21">
+      <c r="I187" s="15"/>
+      <c r="J187" s="15"/>
+      <c r="K187" s="15">
         <v>29.4</v>
       </c>
-      <c r="L187" s="21"/>
-      <c r="M187" s="21"/>
+      <c r="L187" s="15"/>
+      <c r="M187" s="15"/>
     </row>
     <row r="188" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A188" s="2">
@@ -7270,19 +7267,19 @@
       <c r="H188" s="3">
         <v>392.2</v>
       </c>
-      <c r="I188" s="21" t="s">
+      <c r="I188" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J188" s="21">
+      <c r="J188" s="15">
         <v>18.899999999999999</v>
       </c>
-      <c r="K188" s="21">
+      <c r="K188" s="15">
         <v>19.399999999999999</v>
       </c>
-      <c r="L188" s="21">
+      <c r="L188" s="15">
         <v>7.6</v>
       </c>
-      <c r="M188" s="21">
+      <c r="M188" s="15">
         <v>0.32</v>
       </c>
     </row>
@@ -7309,19 +7306,19 @@
       <c r="H189" s="3">
         <v>68.8</v>
       </c>
-      <c r="I189" s="21" t="s">
+      <c r="I189" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J189" s="21">
+      <c r="J189" s="15">
         <v>16.399999999999999</v>
       </c>
-      <c r="K189" s="21">
+      <c r="K189" s="15">
         <v>18.5</v>
       </c>
-      <c r="L189" s="21">
+      <c r="L189" s="15">
         <v>5.8</v>
       </c>
-      <c r="M189" s="21">
+      <c r="M189" s="15">
         <v>0.61</v>
       </c>
     </row>
@@ -7348,19 +7345,19 @@
       <c r="H190" s="3">
         <v>854.7</v>
       </c>
-      <c r="I190" s="21" t="s">
+      <c r="I190" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="J190" s="21">
+      <c r="J190" s="15">
         <v>15.3</v>
       </c>
-      <c r="K190" s="21">
+      <c r="K190" s="15">
         <v>20.2</v>
       </c>
-      <c r="L190" s="21">
+      <c r="L190" s="15">
         <v>6.3330000000000002</v>
       </c>
-      <c r="M190" s="21">
+      <c r="M190" s="15">
         <v>0.69</v>
       </c>
     </row>
@@ -7373,11 +7370,11 @@
       <c r="F191" s="3"/>
       <c r="G191" s="3"/>
       <c r="H191" s="3"/>
-      <c r="I191" s="21"/>
-      <c r="J191" s="21"/>
-      <c r="K191" s="21"/>
-      <c r="L191" s="21"/>
-      <c r="M191" s="21"/>
+      <c r="I191" s="15"/>
+      <c r="J191" s="15"/>
+      <c r="K191" s="15"/>
+      <c r="L191" s="15"/>
+      <c r="M191" s="15"/>
     </row>
     <row r="192" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A192" s="3"/>
@@ -7388,11 +7385,11 @@
       <c r="F192" s="3"/>
       <c r="G192" s="3"/>
       <c r="H192" s="3"/>
-      <c r="I192" s="21"/>
-      <c r="J192" s="21"/>
-      <c r="K192" s="21"/>
-      <c r="L192" s="21"/>
-      <c r="M192" s="21"/>
+      <c r="I192" s="15"/>
+      <c r="J192" s="15"/>
+      <c r="K192" s="15"/>
+      <c r="L192" s="15"/>
+      <c r="M192" s="15"/>
     </row>
     <row r="193" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A193" s="3"/>
@@ -7471,5 +7468,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>